<commit_message>
latest code (exclude large model file >100MB)
</commit_message>
<xml_diff>
--- a/cuisines/Punjabi Cuisines/recipes.xlsx
+++ b/cuisines/Punjabi Cuisines/recipes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,11 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Link to recipe</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Cleaned-Ingredients</t>
         </is>
       </c>
     </row>
@@ -491,6 +496,11 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/saunf-aloo-fennel-potato-curry-recipe</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>fennel seeds (saunf),potato (aloo) skin,milk,red chilli powder,coriander (dhania) leaves,turmeric powder</t>
         </is>
       </c>
     </row>
@@ -537,6 +547,11 @@
           <t>https://www.archanaskitchen.com/baingan-bharta-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>tomato,turmeric powder,salt,ginger,red chilli powder,eggsplant,coriander,onion,oil,coriander powder,green chillies,butter,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -574,6 +589,11 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/makki-and-methi-roti-recipe</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>salt,makki ka atta (yellow corn meal flour),kashmiri red chilli powder,ajwain (carom seeds),methi leaves (fenugreek leaves),green chillies</t>
         </is>
       </c>
     </row>
@@ -617,6 +637,11 @@
           <t>https://www.archanaskitchen.com/maa-ki-dal-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>tomato,salt,ginger,kashmiri red chilli powder,ghee,kidney beans,black urad dal (split),coriander powder,cumin seeds,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -653,6 +678,11 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/dry-masala-chickpeas-recipe-in-hindi</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>turmeric powder,salt,gingerpaste,red chilli powder,kabuli channa soak then boil,spoon cumin powder,amchoor powder,oil,coriander powder,chana masala powder,cumin seeds</t>
         </is>
       </c>
     </row>
@@ -698,6 +728,11 @@
           <t>https://www.archanaskitchen.com/palak-paneer-recipe-cottage-cheese-in-spinach-gravy-in-hindi</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>tomato,turmeric powder,salt,ginger,spinach,paneer,tsp cinnamon powder,cumin powder,cloves garlic,butter,green chillies,cumin seeds,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -737,6 +772,11 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/gur-paare-recipe-a-traditional-punjabi-wedding-sweet</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ghee,fennel seeds (saunf),jaggery,flour (maida),sunflower oil</t>
         </is>
       </c>
     </row>
@@ -779,6 +819,11 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/video-recipe-smoked-tandoori-paneer-tikka</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>salt,cumin powder (jeera),hung curd (greek yogurt),coal coal smoking method,ginger,coriander powder,black salt,paneer,ajwain (carom seeds),saffron strands,cloves garlic,gram flour (besan),onion,fennel seeds (saunf) ground powder,black pepper powder,mint leaves (pudina),turmeric powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -826,6 +871,11 @@
           <t>https://www.archanaskitchen.com/palak-onion-kadhi-pakora-recipe</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>salt,enos fruit salt,hung curd (greek yogurt),green chilli,spinach,asafoetida (hing),ghee,coriander (dhania) leaves,red chilli powder,water,gram flour (besan),curry leaves,onion,cumin seeds (jeera),coriander powder,turmeric powder,garam masala powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -864,6 +914,11 @@
           <t>https://www.archanaskitchen.com/maa-ki-dal-recipe-punjabi-style-slow-cooked-black-urad-lentils</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>tomato,ginger,ghee,kashmiri dry red chillies,black urad dal (split),cumin seeds (jeera),rajma (large kidney beans),coriander powder,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -900,6 +955,11 @@
           <t>https://www.archanaskitchen.com/dry-chole-recipe-dry-masala-chickpeas</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>salt,cumin powder (jeera),coriander powder,amchur (dry mango powder),red chilli powder,kabuli chana (white chickpeas),cumin seeds (jeera),ginger paste,turmeric powder,chana masala powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -933,6 +993,11 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/methi-daana-boondi-kadhi-recipe</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>salt,ghee,asafoetida (hing),red chilli powder,black peppercorns,ginger garlic paste,curd,gram flour (besan),cumin seeds (jeera),methi seeds (fenugreek seeds),turmeric powder,cloves (laung),boondi,green chilli paste</t>
         </is>
       </c>
     </row>
@@ -972,6 +1037,11 @@
           <t>https://www.archanaskitchen.com/tawa-amritsari-kulcha-recipe</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>salt,wheat flour,cumin powder (jeera),green chilli,amchur (dry mango powder),potato (aloo) skin,red chilli powder,curd,turmeric powder,garam masala powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1007,6 +1077,11 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/punjabi-mooli-ki-bhurji-recipe</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>salt,ginger,mustard oil,mooli mullangi (radish) tiny,asafoetida (hing),ajwain (carom seeds),red chilli powder,mooli ke patte (radish greens) (with stem),turmeric powder,green chillies</t>
         </is>
       </c>
     </row>
@@ -1046,6 +1121,11 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/punjabi-wadi-choliya-ki-sabzi-recipe</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>tomato,salt,coriander (dhania),ginger,asafoetida (hing),red chilli powder,curd,green chickpeas,badi (wadi),coriander powder,turmeric powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1093,6 +1173,11 @@
           <t>https://www.archanaskitchen.com/baingan-methi-ka-bharta-recipe-with-pomegranates</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>tomato,salt,ginger,brinjal (baingan eggsplant),anardana powder (pomegranate seed powder),methi leaves (fenugreek leaves),red chilli powder,onion,coriander powder,turmeric powder,green chillies,butter,garam masala powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1133,6 +1218,11 @@
           <t>https://www.archanaskitchen.com/aloo-amritsari-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>tomato,turmeric powder,salt,ginger,kashmiri red chilli powder,onion directly,coriander,celery,spoon garam masala powder,garlic,oil,coriander powder,potatoes</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1168,6 +1258,11 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/rumali-roti-recipe</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>salt,water knead,curd,flour (maida),sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1217,6 +1312,11 @@
           <t>https://www.archanaskitchen.com/kadhi-pakoras-creamy-yogurt-curry-with-fried-dumplings-recipe</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>salt,ginger,water combine the ingredients,ghee,mustard seeds,ajwain (carom seeds),potato (aloo),red chilli powder,water,asafoetida (hing),gram flour (besan),curd,soda,curry leaves,onion,dry red chillies,coriander (dhania) leaves,turmeric powder,green chillies,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1254,6 +1354,11 @@
           <t>https://www.archanaskitchen.com/punjabi-style-lobia-masala-recipe-black-eyed-peas-masala</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>tomato,salt,cumin powder (jeera),fennel seeds (saunf),milk,red chilli powder,ginger garlic paste,sugar,green chillies between,cinnamon stick (dalchini),cumin seeds (jeera),onion,tamarind paste,coriander powder,turmeric powder,black eyed beans (lobia),garam masala powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1283,6 +1388,11 @@
       <c r="F22" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/kasuri-methi-chole-recipe</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>cashew nuts,tomato,salt,bay leaf (tej patta),green chillifor,red chilli powder,kabuli chana (white chickpeas),coriander (dhania) seeds,cinnamon stick (dalchini),cumin seeds (jeera),cloves (laung),turmeric powder,kasuri methi (dried fenugreek leaves),garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1322,6 +1432,11 @@
       <c r="F23" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/lobia-masala-recipe-in-hindi</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>tomato,turmeric powder,cowpea,ginger,salt,green chilli,coriander leaves,red chilli powder,sugar,lemon tamarind water,coriander powder,oil,cumin seeds</t>
         </is>
       </c>
     </row>
@@ -1366,6 +1481,11 @@
           <t>https://www.archanaskitchen.com/rawal-pindi-style-chole-recipe</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>tomato,salt,cumin powder (jeera),ginger,green chilli,amchur (dry mango powder),ghee,anardana powder (pomegranate seed powder),red chilli powder,cloves garlic,kabuli chana (white chickpeas),coriander (dhania) seeds,onion,cumin seeds (jeera),turmeric powder,black tea bag,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1400,6 +1520,11 @@
       <c r="F25" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/punjabi-style-egg-curry-recipe</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>black cardamom (badi elaichi),tomato paste,green chilli,bay leaf (tej patta),cardamom (elaichi) podsseeds,red chilli powder,water,ginger garlic paste,onion paste,coriander (dhania) leaves,onion,coriander powder,eggs,turmeric powder,cloves (laung),garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1439,6 +1564,11 @@
           <t>https://www.archanaskitchen.com/chicken-tariwala-recipe-punjabi-murgh-tariwala-recipe</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>tomato,cumin powder (jeera),cinnamon stick (dalchini) cinnamon,cloves garlic,onion,turmeric powder,green chillies,red chilli paste,sunflower oil,black cardamom (badi elaichi),salt,chicken curry,garam masala powder,star anise,red chilli powder,curd,lemon,ginger,bay leaf (tej patta),coriander powder,cloves (laung)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1475,6 +1605,11 @@
           <t>https://www.archanaskitchen.com/hyderabadi-laziz-lamb-handi-recipe</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>tomato,salt,tomato paste,kashmiri red chilli powder,cumin powder (jeera),coriander powder,ghee,lamb ribs,coriander (dhania) leaves,red chilli powder,water,curd,garlic,onion,lemon,ginger paste,turmeric powder,garam masala powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1508,6 +1643,11 @@
       <c r="F28" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/stuffed-bharwa-tinda-recipe-stuffed-apple-gourd</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>tomato,tinda (apple gourd),cumin powder (jeera),ginger,salt,amchur (dry mango powder),asafoetida (hing),red chilli powder,cloves garlic,coriander (dhania) leaves,onion,coriander powder,turmeric powder,garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1544,6 +1684,11 @@
       <c r="F29" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/makai-wali-bhindi-recipe</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>salt,makki ka atta (yellow corn meal flour),amchur (dry mango powder),red chilli powder,onion,cumin seeds (jeera),bhindi (lady fingerokra),coriander powder,turmeric powder,garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1597,6 +1742,11 @@
           <t>https://www.archanaskitchen.com/kadhi-pakoras-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>potato,kashmiri red chilli powder,onion,green chillies,salt,water mix ingredients,green chilli,mustard,soda,asafoetida,red chilli powder,water,curd cracked,coriander (dhania) leaves finely,oil,turmeric powder,ginger,ghee,celery,curry leaves,gram flour</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1641,6 +1791,11 @@
           <t>https://www.archanaskitchen.com/panjiri-recipe-healthy-punjabi-dry-fruit-snack</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>cashew nuts,wheat flour,nutmeg powder,ghee,pistachios,dry coconut (kopra),chiroti rava,sugar,dry ginger powder,badam (almond),phool makhana (lotus seeds),flax seeds,poppy seeds,cardamom powder (elaichi),gond (natural gum),melon seeds</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1685,6 +1840,11 @@
           <t>https://www.archanaskitchen.com/punjabi-mixed-vegetable-kadai-recipe</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>tomato,cloves garlic,carrot,baby corn,coriander (dhania) seeds,onion,cumin seeds (jeera),turmeric powder,green chillies,salt,cardamom (elaichi) podsseeds,butter oil mixed,garam masala powder,green beans (french beans),cloves cloves (laung),cauliflower (gobi),dry red chilli,sugar,kasuri methi (dried fenugreek leaves),ginger,bay leaf (tej patta),green peas (matar),cinnamon stick (dalchini),green bell pepper (capsicum),potato (aloo)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1718,6 +1878,11 @@
       <c r="F33" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/baked-amritsari-kulcha-recipe-without-yeast</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>salt,baking powder,coriander (dhania) leaves,black sesame seeds,water,baking soda,curd,sugar,flour (maida),sesame seeds (til seeds),butter,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1757,6 +1922,11 @@
           <t>https://www.archanaskitchen.com/chicken-tikka-recipe</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>salt,cumin powder (jeera),boneless chicken,ajwain (carom seeds),red chilli powder,gram flour (besan),ginger garlic paste,curd,lemon,coriander powder,turmeric powder,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1789,6 +1959,11 @@
       <c r="F35" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/aloo-amritsari-recipe</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>tomato,ginger,kashmiri red chilli powder,salt tase,ajwain (carom seeds),cloves garlic,coriander (dhania) leaves,onion,coriander powder,potato (aloo),turmeric powder,garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1840,6 +2015,11 @@
           <t>https://www.archanaskitchen.com/amritsari-chole-recipe-white-chickpeas-in-spicy-gravy</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>tomato,coriander (dhania) leaves,kabuli chana (white chickpeas),coriander (dhania) seeds,onion,turmeric powder,salt,green chilli,dry red chillies,brown cardamom (badi elaichi),tea bags,black pepper corns,methi seeds (fenugreek seeds),dried anardana seeds (pomegranate seeds dried),cumin (jeera) seeds,black salt,ginger,amchur (dry mango powder),ghee,cinnamon stick (dalchini),cloves (laung)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1873,6 +2053,11 @@
       <c r="F37" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/punjabi-style-moth-beans-dal-recipe-matki</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>tomato,salt,ginger,moth dal (matki),green chilli,amchur (dry mango powder),red chilli powder,cloves garlic,onion,cumin seeds (jeera),turmeric powder,garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -1917,6 +2102,11 @@
           <t>https://www.archanaskitchen.com/punjabi-style-arbi-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>turmeric powder,salt,cumin,amchoor,ghee,red chilli powder,coriander,onion,arabic,green chillies,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1951,6 +2141,11 @@
           <t>https://www.archanaskitchen.com/punjabi-style-tinda-sabji-recipe</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>tomato,tinda (apple gourd),cumin powder (jeera),salt,sunflower oil,asafoetida (hing),red chilli powder,cloves garlic,onion,cumin seeds (jeera),coriander powder,turmeric powder,garam masala powder,tomato paste</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1982,6 +2177,11 @@
       <c r="F40" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/mooli-and-wadi-ki-sabzi-recipe</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>salt,mustard oil,mustard seeds,red chilli powder,coriander (dhania) leaves,onion,badi (wadi) punjabi masala,cumin seeds (jeera),turmeric powder,mooli mullangi (radish)</t>
         </is>
       </c>
     </row>
@@ -2016,6 +2216,11 @@
       <c r="F41" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/amritsar-fish-fry-recipe</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>salt,ajwain (carom seeds) pound,amchur (dry mango powder),red chilli powder,ginger garlic paste,gram flour (besan),nutralite classic,lemon,seer fish,turmeric powder,kasuri methi (dried fenugreek leaves),garam masala powder</t>
         </is>
       </c>
     </row>
@@ -2060,6 +2265,11 @@
           <t>https://www.archanaskitchen.com/punjabi-style-egg-curry-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>turmeric powder,green chilli,red chilli powder,ginger garlic paste,onion paste,bay leaf,coriander (dhania) leavestake,onion,oil,cardamom,coriander powder,water used cilantro,eggs,garam masala powder,tomato paste</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2098,6 +2308,11 @@
       <c r="F43" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/punjabi-black-chickpea-curry-recipe-kale-chane-ki-sabzi</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>tomato,salt,garam masala powder,coriander (dhania) leaves,red chilli powder,water,ginger garlic paste,onion,cumin seeds (jeera),kala chana (brown chickpeas),sunflower oil</t>
         </is>
       </c>
     </row>
@@ -2150,6 +2365,11 @@
           <t>https://www.archanaskitchen.com/spiced-indian-potato-flatbread-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>turmeric powder,salt,wheat flour,water make dough,ginger,green chilli,potatoes boil mash karela,cumin powder,coriander (dhania) leaves take mango powder,red chilli powder,onion,coriander powder,oil ghee,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2185,6 +2405,11 @@
       <c r="F45" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/paneer-peshawari-recipe-cottage-cheese-in-rich-gravy</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>tomato,salt,cumin powder (jeera),kashmiri red chilli powder,bay leaf (tej patta),ginger garlic paste,cashews water,onion,cumin seeds (jeera),coriander powder,turmeric powder,kasuri methi (dried fenugreek leaves),butter,garam masala powder,paneer cubes</t>
         </is>
       </c>
     </row>
@@ -2229,6 +2454,11 @@
           <t>https://www.archanaskitchen.com/rajma-and-horse-gram-stuffed-paratha-recipe</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>salt,wheat flour,water knead,green chilli,amchur (dry mango powder),red chilli powder,onion,cumin seeds (jeera),rajma (large kidney beans),black pepper powder,horse gram dal (kollu kulith),coriander powder,garam masala powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2268,6 +2498,11 @@
           <t>https://www.archanaskitchen.com/punjabi-bhindi-kadhi-recipe-roasted-okra-in-yogurt-curry</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>salt,ghee,sunflower oil the bhindi,red chilli powder,gram flour (besan),curd,dry red chillies,cinnamon stick (dalchini),cumin seeds (jeera),coriander powder,bhindi (lady fingerokra) destemmed,turmeric powder</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2303,6 +2538,11 @@
       <c r="F48" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/amritsari-dal-recipe</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>tomato,salt,ginger,chana dal (bengal gram dal),ajwain (carom seeds),red chilli powder,cloves garlic,onion,cinnamon stick (dalchini),black urad dal,green chillies,garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -2345,6 +2585,11 @@
           <t>https://www.archanaskitchen.com/sarson-ka-saag-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>turmeric powder,salt,cheese,ginger,spinach,cumin powder,mustard,batua,garlic,onion,green chilli from the middle,oil,cinnamon powder</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2376,6 +2621,11 @@
       <c r="F50" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/punjabi-choori-recipe-sweet-crumbled-rotis</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>sugar jaggery,mixed nuts like cashew almonds,tawa paratha leftover,ghee</t>
         </is>
       </c>
     </row>
@@ -2420,6 +2670,11 @@
           <t>https://www.archanaskitchen.com/amritsari-dal-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>tomato,turmeric powder,salt,ginger,red chilli powder,lentil sugar,black urad dal (split),chana dal,onion,oil,green chillies,take celery,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2450,6 +2705,11 @@
       <c r="F52" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/fish-tikka-masala-skewer-recipe</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>salt,kashmiri red chilli powder,mustard oil,coriander (dhania) leaves,chaat masala powder,gram flour (besan),curd,fish fillet,lemon,mint leaves (pudina),garam masala powder</t>
         </is>
       </c>
     </row>
@@ -2500,6 +2760,11 @@
           <t>https://www.archanaskitchen.com/smoked-dhaba-dal-recipe</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>tomato,salt,cumin powder (jeera),arhar dal (split toor dal),ginger,green chilli,black salt,ghee,charcoal,red chilli powder,cloves garlic,coriander (dhania) leaves,dry red chillies,onion,cumin seeds (jeera),coriander powder,green moong dal,turmeric powder,sunflower oil</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2533,6 +2798,11 @@
       <c r="F54" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/dal-bukhara-recipe-punjabi-style-black-urad-dal</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>tomato,salt,cumin powder (jeera),chaat masala powder,red chilli powder,ginger garlic paste,onion,cumin seeds (jeera),kasuri methi (dried fenugreek leaves),black urad dal,green chillies,butter,garam masala powder</t>
         </is>
       </c>
     </row>
@@ -2572,6 +2842,11 @@
       <c r="F55" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/amritsari-sookhi-dal-recipe-in-hindi</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>tomato,turmeric powder,ginger,cumin,celery,black urad dal (split),coriander,onion,oil,coriander powder,asafetida,green chillies,coriander leaves finely salt red chilli powder</t>
         </is>
       </c>
     </row>
@@ -2615,6 +2890,11 @@
           <t>https://www.archanaskitchen.com/sarson-ka-saag-a-north-indian-recipe-of-mustard-leaves</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>green chillies,salt,ginger,bathua leaves,makki ka atta (yellow corn meal flour),ghee,red chilli powder,cloves garlic,onion,mustard greens,coriander powder,spinach leaves (palak),garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2649,6 +2929,11 @@
           <t>https://www.archanaskitchen.com/punjabi-style-spicy-arbi-sabji-recipe</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>salt,amchur (dry mango powder),ghee,coriander (dhania) leaves,red chilli powder,colocasia root (arbi),onion,cumin seeds (jeera),turmeric powder,green chillies,garam masala powder</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2679,6 +2964,11 @@
       <c r="F58" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/chatpate-aloo-recipe-with-sesame-seeds</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>salt,cumin powder (jeera),amchur (dry mango powder),coriander (dhania) leaves,red chilli powder,baby potatoes,coriander powder,turmeric powder,sesame seeds (til seeds),garam masala powder,sunflower oil</t>
         </is>
       </c>
     </row>
@@ -2717,6 +3007,11 @@
       <c r="F59" t="inlineStr">
         <is>
           <t>https://www.archanaskitchen.com/hariyali-pav-bhaji-recipe</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>tomato,asafoetida (hing),onion,cumin seeds (jeera),turmeric powder,spinach leaves (palak),sunflower oil,pav bhaji masala,pav buns,green chutney (coriander mint),garam masala powder,mustard seeds,red chilli powder,green chillies(),butter,potato (aloo),green peas (matar),curry leaves,ginger garlic paste,coriander (dhania) leaves,bottle gourd (lauki)</t>
         </is>
       </c>
     </row>
@@ -2764,6 +3059,11 @@
           <t>https://www.archanaskitchen.com/corn-methi-malai-gravy-recipe</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>tomato,amchur (dry mango powder),methi leaves (fenugreek leaves),red chilli powder,black peppercorns,cashews water,sugar,onion,cumin seeds (jeera),cinnamon stick (dalchini),cloves cardamom (elaichi) podsseeds,sweet corn,turmeric powder,cloves (laung),butter</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2802,6 +3102,11 @@
           <t>https://www.archanaskitchen.com/kadai-paneer-recipe-in-hindi</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>cheese,tomato,cardamom powder,ginger,turmeric powder,kasuri methi,salt,capsicum (green),cumin powder,red chilli powder,cloves garlic,onion,oil,black pepper powder,butter</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2836,6 +3141,11 @@
           <t>https://www.archanaskitchen.com/amritsari-sookhi-dal-recipe</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>tomato,salt,ginger,coriander (dhania) leaves,asafoetida (hing),ajwain (carom seeds),red chilli powder,black urad dal (split),onionlengthwise,cumin seeds (jeera),coriander powder,turmeric powder,green chillies,sunflower oil</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>